<commit_message>
fixed missing expected answers
</commit_message>
<xml_diff>
--- a/final_benchmark_with_expected_answers.xlsx
+++ b/final_benchmark_with_expected_answers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7ba8848fe0992bd8/MVP/Blogs/Data Agent Evalutaion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{6880DDB8-E720-434D-B33C-F20C65B8EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E716D5E-98FC-4900-8770-9FB95A3ED500}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{6880DDB8-E720-434D-B33C-F20C65B8EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAD741C4-475E-4390-AFA7-E6A0C0AAF1C4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E0EF22B-6A68-4169-ADB1-AC4A6BF7AAF7}"/>
+    <workbookView xWindow="19090" yWindow="-5130" windowWidth="38620" windowHeight="21100" xr2:uid="{1E0EF22B-6A68-4169-ADB1-AC4A6BF7AAF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="269">
   <si>
     <t>benchmark_split</t>
   </si>
@@ -1012,7 +1012,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="17">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1030,6 +1033,52 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1045,24 +1094,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9430D58F-897A-4A91-B243-3E6A66A0E2FC}" name="Table1" displayName="Table1" ref="A1:O73" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9430D58F-897A-4A91-B243-3E6A66A0E2FC}" name="Table1" displayName="Table1" ref="A1:O73" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A1:O73" xr:uid="{9430D58F-897A-4A91-B243-3E6A66A0E2FC}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{93C2DC27-BFB8-4BA8-9568-12BD122FB24B}" name="benchmark_split"/>
-    <tableColumn id="2" xr3:uid="{D27B7FF8-DD49-41DA-BD27-9D6C6C3594B8}" name="intent_id"/>
-    <tableColumn id="3" xr3:uid="{DF079301-682F-4C41-81F0-C038DC6D7F8F}" name="question_id"/>
-    <tableColumn id="4" xr3:uid="{8DE4D5CE-0155-4EAE-8B54-5A6215E7D3E1}" name="source_type"/>
-    <tableColumn id="5" xr3:uid="{B3246569-20B3-4242-BF4D-072ACB9D704B}" name="language"/>
-    <tableColumn id="6" xr3:uid="{C4D9BCD1-5CDE-4847-A645-5E44395400F1}" name="variant_type"/>
-    <tableColumn id="7" xr3:uid="{BBDB21D7-D078-4BA8-B2A8-F183F2E64241}" name="category_5"/>
-    <tableColumn id="8" xr3:uid="{73CBA146-3E30-43D0-816F-8290D43FFC57}" name="language_sensitivity"/>
-    <tableColumn id="9" xr3:uid="{F6DBE24A-1A52-4FAE-AE3D-78A970F216A2}" name="required_tables"/>
-    <tableColumn id="10" xr3:uid="{ABC14214-AB21-4354-B51A-62C21B2516C0}" name="question"/>
-    <tableColumn id="11" xr3:uid="{B84DFAFD-8E1B-4A97-9FB7-4189A12FA079}" name="expected_answer"/>
-    <tableColumn id="12" xr3:uid="{94DEE702-29B3-4B35-8235-0F20ED40FC26}" name="expected_answer_type"/>
-    <tableColumn id="13" xr3:uid="{7FEA743A-5A41-471D-8AC4-F697958AADBB}" name="comparison_mode"/>
-    <tableColumn id="14" xr3:uid="{CAA3CD8B-B4D3-4DB1-9D98-294519384734}" name="metric_definition"/>
-    <tableColumn id="15" xr3:uid="{7259D11B-C3DC-4D29-9110-72A602D64506}" name="notes"/>
+    <tableColumn id="1" xr3:uid="{93C2DC27-BFB8-4BA8-9568-12BD122FB24B}" name="benchmark_split" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{D27B7FF8-DD49-41DA-BD27-9D6C6C3594B8}" name="intent_id" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{DF079301-682F-4C41-81F0-C038DC6D7F8F}" name="question_id" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{8DE4D5CE-0155-4EAE-8B54-5A6215E7D3E1}" name="source_type" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{B3246569-20B3-4242-BF4D-072ACB9D704B}" name="language" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{C4D9BCD1-5CDE-4847-A645-5E44395400F1}" name="variant_type" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{BBDB21D7-D078-4BA8-B2A8-F183F2E64241}" name="category_5" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{73CBA146-3E30-43D0-816F-8290D43FFC57}" name="language_sensitivity" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{F6DBE24A-1A52-4FAE-AE3D-78A970F216A2}" name="required_tables" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{ABC14214-AB21-4354-B51A-62C21B2516C0}" name="question" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{B84DFAFD-8E1B-4A97-9FB7-4189A12FA079}" name="expected_answer" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{94DEE702-29B3-4B35-8235-0F20ED40FC26}" name="expected_answer_type" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{7FEA743A-5A41-471D-8AC4-F697958AADBB}" name="comparison_mode" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{CAA3CD8B-B4D3-4DB1-9D98-294519384734}" name="metric_definition" dataDxfId="3"/>
+    <tableColumn id="15" xr3:uid="{7259D11B-C3DC-4D29-9110-72A602D64506}" name="notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1454,7 +1503,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="120" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -1501,135 +1550,144 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="L3" t="s">
+      <c r="K3" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="E4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="L4" t="s">
+      <c r="K4" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="E5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="L5" t="s">
+      <c r="K5" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O5" s="3" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1680,135 +1738,144 @@
         <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:15" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="E7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="L7" t="s">
+      <c r="K7" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O7" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:15" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="E8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L8" t="s">
+      <c r="K8" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="O8" t="s">
+      <c r="O8" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:15" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="E9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="L9" t="s">
+      <c r="K9" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O9" s="3" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1859,135 +1926,144 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="L11" t="s">
+      <c r="K11" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N11" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="O11" t="s">
+      <c r="O11" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="E12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="L12" t="s">
+      <c r="K12" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N12" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O12" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E13" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="E13" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="L13" t="s">
+      <c r="K13" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="L13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N13" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="O13" t="s">
+      <c r="O13" s="3" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2038,135 +2114,144 @@
         <v>101</v>
       </c>
     </row>
-    <row r="15" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:15" ht="330" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E15" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="E15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="L15" t="s">
+      <c r="K15" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="N15" t="s">
+      <c r="N15" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="O15" t="s">
+      <c r="O15" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:15" ht="330" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E16" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="E16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="L16" t="s">
+      <c r="K16" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="L16" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="O16" t="s">
+      <c r="O16" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="17" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:15" ht="330" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E17" t="s">
-        <v>50</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="E17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="L17" t="s">
+      <c r="K17" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="N17" t="s">
+      <c r="N17" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="O17" t="s">
+      <c r="O17" s="3" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2217,135 +2302,144 @@
         <v>114</v>
       </c>
     </row>
-    <row r="19" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E19" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E19" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="L19" t="s">
+      <c r="K19" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="L19" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N19" t="s">
+      <c r="N19" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="3" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E20" t="s">
-        <v>50</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="E20" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="L20" t="s">
+      <c r="K20" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N20" t="s">
+      <c r="N20" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="O20" t="s">
+      <c r="O20" s="3" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E21" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="E21" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="L21" t="s">
+      <c r="K21" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M21" t="s">
+      <c r="M21" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N21" t="s">
+      <c r="N21" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="O21" t="s">
+      <c r="O21" s="3" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2396,135 +2490,144 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D23" t="s">
-        <v>121</v>
-      </c>
-      <c r="E23" t="s">
-        <v>50</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="D23" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="L23" t="s">
+      <c r="K23" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M23" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N23" t="s">
+      <c r="N23" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O23" t="s">
+      <c r="O23" s="3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" t="s">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D24" t="s">
-        <v>121</v>
-      </c>
-      <c r="E24" t="s">
-        <v>50</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="D24" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="L24" t="s">
+      <c r="K24" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M24" t="s">
+      <c r="M24" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N24" t="s">
+      <c r="N24" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O24" t="s">
+      <c r="O24" s="3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" t="s">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D25" t="s">
-        <v>121</v>
-      </c>
-      <c r="E25" t="s">
-        <v>50</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="D25" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="L25" t="s">
+      <c r="K25" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M25" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N25" t="s">
+      <c r="N25" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O25" t="s">
+      <c r="O25" s="3" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2575,135 +2678,144 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="27" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D27" t="s">
-        <v>121</v>
-      </c>
-      <c r="E27" t="s">
-        <v>50</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="D27" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="L27" t="s">
+      <c r="K27" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="L27" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M27" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N27" t="s">
+      <c r="N27" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O27" t="s">
+      <c r="O27" s="3" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" t="s">
+    <row r="28" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="D28" t="s">
-        <v>121</v>
-      </c>
-      <c r="E28" t="s">
-        <v>50</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="D28" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="L28" t="s">
+      <c r="K28" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="L28" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M28" t="s">
+      <c r="M28" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N28" t="s">
+      <c r="N28" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O28" t="s">
+      <c r="O28" s="3" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="29" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="29" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D29" t="s">
-        <v>121</v>
-      </c>
-      <c r="E29" t="s">
-        <v>50</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="D29" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="L29" t="s">
+      <c r="K29" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="L29" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M29" t="s">
+      <c r="M29" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N29" t="s">
+      <c r="N29" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O29" t="s">
+      <c r="O29" s="3" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2754,135 +2866,144 @@
         <v>145</v>
       </c>
     </row>
-    <row r="31" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" t="s">
+    <row r="31" spans="1:15" ht="225" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D31" t="s">
-        <v>121</v>
-      </c>
-      <c r="E31" t="s">
-        <v>50</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="D31" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="L31" t="s">
+      <c r="K31" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="L31" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M31" t="s">
+      <c r="M31" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N31" t="s">
+      <c r="N31" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O31" t="s">
+      <c r="O31" s="3" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="32" spans="1:15" ht="225" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D32" t="s">
-        <v>121</v>
-      </c>
-      <c r="E32" t="s">
-        <v>50</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="D32" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="L32" t="s">
+      <c r="K32" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="L32" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M32" t="s">
+      <c r="M32" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N32" t="s">
+      <c r="N32" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O32" t="s">
+      <c r="O32" s="3" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" t="s">
+    <row r="33" spans="1:15" ht="225" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D33" t="s">
-        <v>121</v>
-      </c>
-      <c r="E33" t="s">
-        <v>50</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="D33" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H33" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J33" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="L33" t="s">
+      <c r="K33" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="L33" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M33" t="s">
+      <c r="M33" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N33" t="s">
+      <c r="N33" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O33" t="s">
+      <c r="O33" s="3" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2933,135 +3054,144 @@
         <v>155</v>
       </c>
     </row>
-    <row r="35" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>20</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="35" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D35" t="s">
-        <v>121</v>
-      </c>
-      <c r="E35" t="s">
-        <v>50</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="D35" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J35" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="L35" t="s">
+      <c r="K35" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="L35" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="M35" t="s">
+      <c r="M35" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="N35" t="s">
+      <c r="N35" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O35" t="s">
+      <c r="O35" s="3" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="36" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" t="s">
+    <row r="36" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D36" t="s">
-        <v>121</v>
-      </c>
-      <c r="E36" t="s">
-        <v>50</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="D36" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J36" t="s">
+      <c r="J36" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="L36" t="s">
+      <c r="K36" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="L36" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="M36" t="s">
+      <c r="M36" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="N36" t="s">
+      <c r="N36" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O36" t="s">
+      <c r="O36" s="3" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="37" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" t="s">
+    <row r="37" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D37" t="s">
-        <v>121</v>
-      </c>
-      <c r="E37" t="s">
-        <v>50</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="D37" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H37" t="s">
+      <c r="H37" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J37" t="s">
+      <c r="J37" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="L37" t="s">
+      <c r="K37" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="L37" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="M37" t="s">
+      <c r="M37" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="N37" t="s">
+      <c r="N37" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="O37" t="s">
+      <c r="O37" s="3" t="s">
         <v>155</v>
       </c>
     </row>
@@ -3112,139 +3242,148 @@
         <v>165</v>
       </c>
     </row>
-    <row r="39" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>20</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="39" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D39" t="s">
-        <v>121</v>
-      </c>
-      <c r="E39" t="s">
-        <v>50</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="D39" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H39" t="s">
+      <c r="H39" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J39" t="s">
+      <c r="J39" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="L39" t="s">
+      <c r="K39" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="L39" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M39" t="s">
+      <c r="M39" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N39" t="s">
+      <c r="N39" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="O39" t="s">
+      <c r="O39" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="40" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>20</v>
-      </c>
-      <c r="B40" t="s">
+    <row r="40" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D40" t="s">
-        <v>121</v>
-      </c>
-      <c r="E40" t="s">
-        <v>50</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="D40" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H40" t="s">
+      <c r="H40" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="L40" t="s">
+      <c r="K40" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="L40" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M40" t="s">
+      <c r="M40" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N40" t="s">
+      <c r="N40" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="O40" t="s">
+      <c r="O40" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="41" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" t="s">
+    <row r="41" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D41" t="s">
-        <v>121</v>
-      </c>
-      <c r="E41" t="s">
-        <v>50</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="D41" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G41" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H41" t="s">
+      <c r="H41" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I41" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J41" t="s">
+      <c r="J41" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="L41" t="s">
+      <c r="K41" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="L41" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="M41" t="s">
+      <c r="M41" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N41" t="s">
+      <c r="N41" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="O41" t="s">
+      <c r="O41" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>20</v>
       </c>
@@ -3291,135 +3430,144 @@
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" t="s">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D43" t="s">
-        <v>121</v>
-      </c>
-      <c r="E43" t="s">
-        <v>50</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="D43" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H43" t="s">
+      <c r="H43" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I43" t="s">
+      <c r="I43" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="J43" t="s">
+      <c r="J43" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="L43" t="s">
+      <c r="K43" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="L43" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M43" t="s">
+      <c r="M43" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N43" t="s">
+      <c r="N43" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O43" t="s">
+      <c r="O43" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" t="s">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="D44" t="s">
-        <v>121</v>
-      </c>
-      <c r="E44" t="s">
-        <v>50</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="D44" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G44" t="s">
+      <c r="G44" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H44" t="s">
+      <c r="H44" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I44" t="s">
+      <c r="I44" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="L44" t="s">
+      <c r="K44" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="L44" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M44" t="s">
+      <c r="M44" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N44" t="s">
+      <c r="N44" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O44" t="s">
+      <c r="O44" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="45" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>20</v>
-      </c>
-      <c r="B45" t="s">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D45" t="s">
-        <v>121</v>
-      </c>
-      <c r="E45" t="s">
-        <v>50</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="D45" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G45" t="s">
+      <c r="G45" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H45" t="s">
+      <c r="H45" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J45" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="L45" t="s">
+      <c r="K45" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="L45" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M45" t="s">
+      <c r="M45" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N45" t="s">
+      <c r="N45" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O45" t="s">
+      <c r="O45" s="3" t="s">
         <v>175</v>
       </c>
     </row>
@@ -3470,139 +3618,148 @@
         <v>184</v>
       </c>
     </row>
-    <row r="47" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>20</v>
-      </c>
-      <c r="B47" t="s">
+    <row r="47" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="D47" t="s">
-        <v>121</v>
-      </c>
-      <c r="E47" t="s">
-        <v>50</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="D47" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G47" t="s">
+      <c r="G47" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H47" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I47" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J47" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="L47" t="s">
+      <c r="K47" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="L47" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M47" t="s">
+      <c r="M47" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N47" t="s">
+      <c r="N47" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="O47" t="s">
+      <c r="O47" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="48" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>20</v>
-      </c>
-      <c r="B48" t="s">
+    <row r="48" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D48" t="s">
-        <v>121</v>
-      </c>
-      <c r="E48" t="s">
-        <v>50</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="D48" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G48" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H48" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="L48" t="s">
+      <c r="K48" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="L48" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M48" t="s">
+      <c r="M48" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N48" t="s">
+      <c r="N48" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="O48" t="s">
+      <c r="O48" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>20</v>
-      </c>
-      <c r="B49" t="s">
+    <row r="49" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D49" t="s">
-        <v>121</v>
-      </c>
-      <c r="E49" t="s">
-        <v>50</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="D49" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G49" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H49" t="s">
+      <c r="H49" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I49" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J49" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="L49" t="s">
+      <c r="K49" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="L49" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="M49" t="s">
+      <c r="M49" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="N49" t="s">
+      <c r="N49" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="O49" t="s">
+      <c r="O49" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -3649,135 +3806,144 @@
         <v>193</v>
       </c>
     </row>
-    <row r="51" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>20</v>
-      </c>
-      <c r="B51" t="s">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="D51" t="s">
-        <v>121</v>
-      </c>
-      <c r="E51" t="s">
-        <v>50</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="D51" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F51" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G51" t="s">
+      <c r="G51" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H51" t="s">
+      <c r="H51" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I51" t="s">
+      <c r="I51" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J51" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="L51" t="s">
+      <c r="K51" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="L51" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M51" t="s">
+      <c r="M51" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N51" t="s">
+      <c r="N51" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O51" t="s">
+      <c r="O51" s="3" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="52" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>20</v>
-      </c>
-      <c r="B52" t="s">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D52" t="s">
-        <v>121</v>
-      </c>
-      <c r="E52" t="s">
-        <v>50</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="D52" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F52" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G52" t="s">
+      <c r="G52" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H52" t="s">
+      <c r="H52" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I52" t="s">
+      <c r="I52" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J52" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="L52" t="s">
+      <c r="K52" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="L52" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M52" t="s">
+      <c r="M52" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N52" t="s">
+      <c r="N52" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O52" t="s">
+      <c r="O52" s="3" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="53" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>20</v>
-      </c>
-      <c r="B53" t="s">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D53" t="s">
-        <v>121</v>
-      </c>
-      <c r="E53" t="s">
-        <v>50</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="D53" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F53" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G53" t="s">
+      <c r="G53" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H53" t="s">
+      <c r="H53" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I53" t="s">
+      <c r="I53" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J53" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="L53" t="s">
+      <c r="K53" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="L53" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="M53" t="s">
+      <c r="M53" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N53" t="s">
+      <c r="N53" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O53" t="s">
+      <c r="O53" s="3" t="s">
         <v>193</v>
       </c>
     </row>
@@ -3828,144 +3994,144 @@
         <v>204</v>
       </c>
     </row>
-    <row r="55" spans="1:15" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" t="s">
+    <row r="55" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D55" t="s">
-        <v>121</v>
-      </c>
-      <c r="E55" t="s">
-        <v>50</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="D55" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G55" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H55" t="s">
+      <c r="H55" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I55" t="s">
+      <c r="I55" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J55" t="s">
+      <c r="J55" s="3" t="s">
         <v>206</v>
       </c>
       <c r="K55" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="L55" t="s">
+      <c r="L55" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="M55" t="s">
+      <c r="M55" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="N55" t="s">
+      <c r="N55" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O55" t="s">
+      <c r="O55" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="56" spans="1:15" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>20</v>
-      </c>
-      <c r="B56" t="s">
+    <row r="56" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D56" t="s">
-        <v>121</v>
-      </c>
-      <c r="E56" t="s">
-        <v>50</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="D56" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F56" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G56" t="s">
+      <c r="G56" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H56" t="s">
+      <c r="H56" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I56" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J56" s="3" t="s">
         <v>208</v>
       </c>
       <c r="K56" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="L56" t="s">
+      <c r="L56" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="M56" t="s">
+      <c r="M56" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="N56" t="s">
+      <c r="N56" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O56" t="s">
+      <c r="O56" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="57" spans="1:15" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>20</v>
-      </c>
-      <c r="B57" t="s">
+    <row r="57" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="D57" t="s">
-        <v>121</v>
-      </c>
-      <c r="E57" t="s">
-        <v>50</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="D57" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G57" t="s">
+      <c r="G57" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H57" t="s">
+      <c r="H57" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I57" t="s">
+      <c r="I57" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J57" s="3" t="s">
         <v>210</v>
       </c>
       <c r="K57" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="L57" t="s">
+      <c r="L57" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="M57" t="s">
+      <c r="M57" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="N57" t="s">
+      <c r="N57" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O57" t="s">
+      <c r="O57" s="3" t="s">
         <v>204</v>
       </c>
     </row>
@@ -4016,144 +4182,144 @@
         <v>215</v>
       </c>
     </row>
-    <row r="59" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>20</v>
-      </c>
-      <c r="B59" t="s">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="D59" t="s">
-        <v>121</v>
-      </c>
-      <c r="E59" t="s">
-        <v>50</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="D59" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G59" t="s">
+      <c r="G59" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H59" t="s">
+      <c r="H59" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I59" t="s">
+      <c r="I59" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J59" s="3" t="s">
         <v>217</v>
       </c>
       <c r="K59" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="L59" t="s">
+      <c r="L59" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="M59" t="s">
+      <c r="M59" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="N59" t="s">
+      <c r="N59" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="O59" t="s">
+      <c r="O59" s="3" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="60" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>20</v>
-      </c>
-      <c r="B60" t="s">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D60" t="s">
-        <v>121</v>
-      </c>
-      <c r="E60" t="s">
-        <v>50</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="D60" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F60" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G60" t="s">
+      <c r="G60" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H60" t="s">
+      <c r="H60" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I60" t="s">
+      <c r="I60" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J60" s="3" t="s">
         <v>219</v>
       </c>
       <c r="K60" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="L60" t="s">
+      <c r="L60" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="M60" t="s">
+      <c r="M60" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="N60" t="s">
+      <c r="N60" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="O60" t="s">
+      <c r="O60" s="3" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="61" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>20</v>
-      </c>
-      <c r="B61" t="s">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C61" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="D61" t="s">
-        <v>121</v>
-      </c>
-      <c r="E61" t="s">
-        <v>50</v>
-      </c>
-      <c r="F61" t="s">
+      <c r="D61" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G61" t="s">
+      <c r="G61" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H61" t="s">
+      <c r="H61" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I61" t="s">
+      <c r="I61" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J61" s="3" t="s">
         <v>221</v>
       </c>
       <c r="K61" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="L61" t="s">
+      <c r="L61" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="M61" t="s">
+      <c r="M61" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="N61" t="s">
+      <c r="N61" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="O61" t="s">
+      <c r="O61" s="3" t="s">
         <v>215</v>
       </c>
     </row>
@@ -4204,148 +4370,148 @@
         <v>224</v>
       </c>
     </row>
-    <row r="63" spans="1:15" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>20</v>
-      </c>
-      <c r="B63" t="s">
+    <row r="63" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B63" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D63" t="s">
-        <v>121</v>
-      </c>
-      <c r="E63" t="s">
-        <v>50</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="D63" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F63" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G63" t="s">
+      <c r="G63" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="H63" t="s">
+      <c r="H63" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I63" t="s">
+      <c r="I63" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J63" t="s">
+      <c r="J63" s="3" t="s">
         <v>226</v>
       </c>
       <c r="K63" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="L63" t="s">
+      <c r="L63" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M63" t="s">
+      <c r="M63" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N63" t="s">
+      <c r="N63" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O63" t="s">
+      <c r="O63" s="3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="64" spans="1:15" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>20</v>
-      </c>
-      <c r="B64" t="s">
+    <row r="64" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="D64" t="s">
-        <v>121</v>
-      </c>
-      <c r="E64" t="s">
-        <v>50</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="D64" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F64" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G64" t="s">
+      <c r="G64" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="H64" t="s">
+      <c r="H64" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I64" t="s">
+      <c r="I64" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J64" s="3" t="s">
         <v>228</v>
       </c>
       <c r="K64" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="L64" t="s">
+      <c r="L64" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M64" t="s">
+      <c r="M64" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N64" t="s">
+      <c r="N64" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O64" t="s">
+      <c r="O64" s="3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="65" spans="1:15" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>20</v>
-      </c>
-      <c r="B65" t="s">
+    <row r="65" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C65" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="D65" t="s">
-        <v>121</v>
-      </c>
-      <c r="E65" t="s">
-        <v>50</v>
-      </c>
-      <c r="F65" t="s">
+      <c r="D65" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F65" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G65" t="s">
+      <c r="G65" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="H65" t="s">
+      <c r="H65" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I65" t="s">
+      <c r="I65" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="J65" t="s">
+      <c r="J65" s="3" t="s">
         <v>230</v>
       </c>
       <c r="K65" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="L65" t="s">
+      <c r="L65" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="M65" t="s">
+      <c r="M65" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N65" t="s">
+      <c r="N65" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O65" t="s">
+      <c r="O65" s="3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>20</v>
       </c>
@@ -4392,144 +4558,144 @@
         <v>233</v>
       </c>
     </row>
-    <row r="67" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>20</v>
-      </c>
-      <c r="B67" t="s">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B67" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="D67" t="s">
-        <v>121</v>
-      </c>
-      <c r="E67" t="s">
-        <v>50</v>
-      </c>
-      <c r="F67" t="s">
+      <c r="D67" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G67" t="s">
+      <c r="G67" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H67" t="s">
+      <c r="H67" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I67" t="s">
+      <c r="I67" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J67" t="s">
+      <c r="J67" s="3" t="s">
         <v>235</v>
       </c>
       <c r="K67" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="L67" t="s">
+      <c r="L67" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="M67" t="s">
+      <c r="M67" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="N67" t="s">
+      <c r="N67" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O67" t="s">
+      <c r="O67" s="3" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="68" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>20</v>
-      </c>
-      <c r="B68" t="s">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="D68" t="s">
-        <v>121</v>
-      </c>
-      <c r="E68" t="s">
-        <v>50</v>
-      </c>
-      <c r="F68" t="s">
+      <c r="D68" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G68" t="s">
+      <c r="G68" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H68" t="s">
+      <c r="H68" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I68" t="s">
+      <c r="I68" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J68" t="s">
+      <c r="J68" s="3" t="s">
         <v>237</v>
       </c>
       <c r="K68" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="L68" t="s">
+      <c r="L68" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="M68" t="s">
+      <c r="M68" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="N68" t="s">
+      <c r="N68" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O68" t="s">
+      <c r="O68" s="3" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="69" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>20</v>
-      </c>
-      <c r="B69" t="s">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D69" t="s">
-        <v>121</v>
-      </c>
-      <c r="E69" t="s">
-        <v>50</v>
-      </c>
-      <c r="F69" t="s">
+      <c r="D69" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G69" t="s">
+      <c r="G69" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H69" t="s">
+      <c r="H69" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I69" t="s">
+      <c r="I69" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J69" t="s">
+      <c r="J69" s="3" t="s">
         <v>239</v>
       </c>
       <c r="K69" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="L69" t="s">
+      <c r="L69" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="M69" t="s">
+      <c r="M69" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="N69" t="s">
+      <c r="N69" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O69" t="s">
+      <c r="O69" s="3" t="s">
         <v>233</v>
       </c>
     </row>
@@ -4580,144 +4746,144 @@
         <v>244</v>
       </c>
     </row>
-    <row r="71" spans="1:15" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>20</v>
-      </c>
-      <c r="B71" t="s">
+    <row r="71" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D71" t="s">
-        <v>121</v>
-      </c>
-      <c r="E71" t="s">
-        <v>50</v>
-      </c>
-      <c r="F71" t="s">
+      <c r="D71" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G71" t="s">
+      <c r="G71" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H71" t="s">
+      <c r="H71" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I71" t="s">
+      <c r="I71" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J71" t="s">
+      <c r="J71" s="3" t="s">
         <v>246</v>
       </c>
       <c r="K71" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="L71" t="s">
+      <c r="L71" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="M71" t="s">
+      <c r="M71" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N71" t="s">
+      <c r="N71" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O71" t="s">
+      <c r="O71" s="3" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="72" spans="1:15" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>20</v>
-      </c>
-      <c r="B72" t="s">
+    <row r="72" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B72" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="D72" t="s">
-        <v>121</v>
-      </c>
-      <c r="E72" t="s">
-        <v>50</v>
-      </c>
-      <c r="F72" t="s">
+      <c r="D72" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F72" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G72" t="s">
+      <c r="G72" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H72" t="s">
+      <c r="H72" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I72" t="s">
+      <c r="I72" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J72" t="s">
+      <c r="J72" s="3" t="s">
         <v>248</v>
       </c>
       <c r="K72" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="L72" t="s">
+      <c r="L72" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="M72" t="s">
+      <c r="M72" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N72" t="s">
+      <c r="N72" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O72" t="s">
+      <c r="O72" s="3" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="73" spans="1:15" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>20</v>
-      </c>
-      <c r="B73" t="s">
+    <row r="73" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B73" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="D73" t="s">
-        <v>121</v>
-      </c>
-      <c r="E73" t="s">
-        <v>50</v>
-      </c>
-      <c r="F73" t="s">
+      <c r="D73" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F73" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G73" t="s">
+      <c r="G73" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H73" t="s">
+      <c r="H73" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I73" t="s">
+      <c r="I73" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J73" t="s">
+      <c r="J73" s="3" t="s">
         <v>250</v>
       </c>
       <c r="K73" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="L73" t="s">
+      <c r="L73" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="M73" t="s">
+      <c r="M73" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="N73" t="s">
+      <c r="N73" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O73" t="s">
+      <c r="O73" s="3" t="s">
         <v>244</v>
       </c>
     </row>

</xml_diff>